<commit_message>
Deployed df854b850 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C349"/>
+  <dimension ref="A1:C326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,7 +494,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'GeoBC TRIM Program' in DataCite not found in CKAN record</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'TRIM BC Base Annotations data' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'GeoBC TRIM Program' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'TRIM BC Base Annotations data' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0272fd06-6ac8-48cd-80c9-b6e05f15be0f</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>0272fd06-6ac8-48cd-80c9-b6e05f15be0f</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>No publisher</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -839,12 +839,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -869,12 +869,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/1.566666' (IsVersionOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://npafc.org/wp-content/uploads/Public-Documents/2018/1790Canada.pdf' (IsSourceOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/1.566666' (IsVersionOf) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://npafc.org/wp-content/uploads/Public-Documents/2018/1790Canada.pdf' (IsSourceOf) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -944,12 +944,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -974,12 +974,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1034,12 +1034,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://hakai-segmentation.readthedocs.io/en/latest/' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://hakai-segmentation.readthedocs.io/en/latest/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>328b062b-3af6-4149-b90f-a85b99dc40eb</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>328b062b-3af6-4149-b90f-a85b99dc40eb</t>
+          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://10.21966/5n09-aq76' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/5n09-aq76' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/5n09-aq76' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/5n09-aq76' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Drew Jordison' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Drew Jordison' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Alex Hare' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Alex Hare' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: title CKAN='High-resolution time series of surface seawater CO2 content from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA' | DataCite='High-resolution record of surface seawater CO2 content from 2016-08 to 2019-05 from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA (NCEI Accession 0246099)'</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>No publisher</t>
+          <t>Metadata mismatch: creator 'Katie Pocock' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Katie Campbell' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.25921/kmam-ct93' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.21966/pk18-z035' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1784,12 +1784,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>No publisher</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2084,12 +2084,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2129,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2159,12 +2159,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2174,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2189,12 +2189,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.48321/d1ae4278b4' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2234,12 +2234,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d1ae4278b4' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2249,12 +2249,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2294,12 +2294,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_jsp' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -2339,12 +2339,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>582c6ff0-029e-44ba-8ba1-d3f2f39f2005</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.21966/1.566666' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2399,12 +2399,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_jsp' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1002/lno.11538' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2414,12 +2414,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>582c6ff0-029e-44ba-8ba1-d3f2f39f2005</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/1.566666' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -2444,12 +2444,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/lno.11538' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2459,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -2489,12 +2489,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2519,12 +2519,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2549,12 +2549,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -2564,12 +2564,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2579,12 +2579,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2639,12 +2639,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
         </is>
       </c>
     </row>
@@ -2654,12 +2654,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2669,12 +2669,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2714,12 +2714,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2729,12 +2729,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2744,12 +2744,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
         </is>
       </c>
     </row>
@@ -2759,12 +2759,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://10.21966/cqrt-sk09' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2774,12 +2774,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2789,12 +2789,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/cqrt-sk09' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2819,12 +2819,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2834,12 +2834,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/1.566666' (Continues) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2849,12 +2849,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.14288/1.0396439' (IsSourceOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -2879,12 +2879,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/1.566666' (Continues) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2894,12 +2894,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.14288/1.0396439' (IsSourceOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2909,12 +2909,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2939,12 +2939,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2969,12 +2969,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2984,12 +2984,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2999,12 +2999,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -3014,12 +3014,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3029,12 +3029,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3049,7 +3049,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3059,12 +3059,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3074,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -3104,12 +3104,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3119,12 +3119,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
+          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3134,7 +3134,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -3149,12 +3149,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3164,12 +3164,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3194,12 +3194,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3224,12 +3224,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3239,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3254,12 +3254,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3269,12 +3269,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3284,12 +3284,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3299,12 +3299,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3314,12 +3314,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3334,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3344,12 +3344,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3359,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -3389,12 +3389,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3404,12 +3404,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3419,7 +3419,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -3434,12 +3434,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3449,12 +3449,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>No publisher</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3464,12 +3464,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Katie Campbell' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.21966/m5rv-4f16' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Wiley Evans' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3494,12 +3494,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Alex Hare' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3509,12 +3509,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Carrie Weekes' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3524,12 +3524,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3539,12 +3539,12 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3554,12 +3554,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3569,12 +3569,12 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>No publisher</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3584,12 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3599,12 +3599,12 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -3614,12 +3614,12 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3629,12 +3629,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3644,12 +3644,12 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/m5rv-4f16' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3659,12 +3659,12 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3674,12 +3674,12 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3689,12 +3689,12 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3704,12 +3704,12 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3719,12 +3719,12 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>a9527050-a108-46f7-ac9f-7150b4abede5</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3734,12 +3734,12 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>a9527050-a108-46f7-ac9f-7150b4abede5</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://10.21966/xp9x-m243' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3749,12 +3749,12 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>a9527050-a108-46f7-ac9f-7150b4abede5</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3764,12 +3764,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>a9527050-a108-46f7-ac9f-7150b4abede5</t>
+          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>No publisher</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3779,12 +3779,12 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: version CKAN='2.1.0' | DataCite='2.0'</t>
         </is>
       </c>
     </row>
@@ -3794,12 +3794,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3809,12 +3809,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3824,12 +3824,12 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3839,12 +3839,12 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Emily Haughton' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3854,12 +3854,12 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Isabelle Desmarais' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3869,12 +3869,12 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Robert White' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -3899,12 +3899,12 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3914,12 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3929,12 +3929,12 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3944,12 +3944,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3959,12 +3959,12 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/xp9x-m243' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3974,12 +3974,12 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -4004,12 +4004,12 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4019,12 +4019,12 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4034,12 +4034,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>2dd906f9-e0fe-4b8c-afe6-c5f2bf7400ae</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Emily Haughton' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -4049,12 +4049,12 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Isabelle Desmarais' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4064,12 +4064,12 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Robert White' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/4kr2-jc55' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4079,12 +4079,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.1.0' | DataCite='2.0'</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4094,12 +4094,12 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4109,12 +4109,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -4124,12 +4124,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4139,12 +4139,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2dd906f9-e0fe-4b8c-afe6-c5f2bf7400ae</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4154,12 +4154,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4169,12 +4169,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4184,12 +4184,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/t8hm-ge90' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4199,12 +4199,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/t8hm-ge90' (Continues) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -4229,12 +4229,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -4244,12 +4244,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -4259,12 +4259,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -4274,12 +4274,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4289,12 +4289,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/4kr2-jc55' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -4304,12 +4304,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4319,12 +4319,12 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>Metadata mismatch: author 'William C. Floyd' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4334,12 +4334,12 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'A. A. Oliver' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4349,7 +4349,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -4364,12 +4364,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4379,12 +4379,12 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4394,12 +4394,12 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4409,12 +4409,12 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/t8hm-ge90' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4424,12 +4424,12 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/t8hm-ge90' (Continues) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4439,7 +4439,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
+          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -4454,12 +4454,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4469,12 +4469,12 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Maartje C. Korver' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4484,12 +4484,12 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'William C. Floyd' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4499,12 +4499,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>15f1d4a2-c82a-450c-a8f7-badb34b9c0dc</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Ray Brunsting' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4514,12 +4514,12 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>15f1d4a2-c82a-450c-a8f7-badb34b9c0dc</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4529,12 +4529,12 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>15f1d4a2-c82a-450c-a8f7-badb34b9c0dc</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>No publisher</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -4544,12 +4544,12 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4559,12 +4559,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'William C. Floyd' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/ytgc-6g46' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4574,12 +4574,12 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'A. A. Oliver' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/zjc2-b004' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4589,12 +4589,12 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/ytgc-6g46' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4604,12 +4604,12 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4619,12 +4619,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4634,12 +4634,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4649,12 +4649,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4664,12 +4664,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4679,12 +4679,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4694,12 +4694,12 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4709,12 +4709,12 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4724,12 +4724,12 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4739,12 +4739,12 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4754,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -4784,12 +4784,12 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4799,12 +4799,12 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/zjc2-b004' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4814,12 +4814,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/ytgc-6g46' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -4829,12 +4829,12 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/zjc2-b004' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -4844,12 +4844,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/ytgc-6g46' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -4859,12 +4859,12 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -4874,12 +4874,12 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Maartje C. Korver' in CKAN record not found in DataCite</t>
+          <t>Contact missing ORCID: Korver, Maartje</t>
         </is>
       </c>
     </row>
@@ -4889,12 +4889,12 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'William C. Floyd' in CKAN record not found in DataCite</t>
+          <t>Contact missing ORCID: Oliver, Allison A.</t>
         </is>
       </c>
     </row>
@@ -4904,12 +4904,12 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Ray Brunsting' in CKAN record not found in DataCite</t>
+          <t>Contact missing ORCID: Janusson, Carly</t>
         </is>
       </c>
     </row>
@@ -4919,12 +4919,12 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing ORCID: Hare, Alex</t>
         </is>
       </c>
     </row>
@@ -4934,12 +4934,12 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Contact missing ORCID: Giesbrecht, Ian</t>
         </is>
       </c>
     </row>
@@ -4949,12 +4949,12 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Contact missing ORCID: Menounos, Brian</t>
         </is>
       </c>
     </row>
@@ -4964,12 +4964,12 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>a8f61379-14f9-4ccc-bc9b-4408ba8340d7</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
+          <t>Contact missing ORCID: Opie, Rumer</t>
         </is>
       </c>
     </row>
@@ -4979,12 +4979,12 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>c06cb551-351c-456f-8d0c-c8aab9aec162</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Contact missing ORCID: Oliver, Allison A.</t>
         </is>
       </c>
     </row>
@@ -4994,12 +4994,12 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Contact missing ORCID: Godwin, Sean</t>
         </is>
       </c>
     </row>
@@ -5009,12 +5009,12 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Contact missing ORCID: Krkosek, Martin</t>
         </is>
       </c>
     </row>
@@ -5024,12 +5024,12 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Contact missing ORCID: Rogers, Luke A.</t>
         </is>
       </c>
     </row>
@@ -5039,12 +5039,12 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Contact missing ORCID: McInnes, Will</t>
         </is>
       </c>
     </row>
@@ -5054,12 +5054,12 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing ORCID: Savage, Rosie</t>
         </is>
       </c>
     </row>
@@ -5069,12 +5069,12 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
+          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing ORCID: Hunt, Brian</t>
         </is>
       </c>
     </row>
@@ -5084,12 +5084,12 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
+          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Contact missing ORCID: Haughton, Emily</t>
         </is>
       </c>
     </row>
@@ -5099,12 +5099,12 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Contact missing ORCID: Korver, Maartje</t>
         </is>
       </c>
     </row>
@@ -5114,12 +5114,12 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
+          <t>Contact missing ORCID: Holmes, Keith</t>
         </is>
       </c>
     </row>
@@ -5129,12 +5129,12 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
+          <t>Contact missing ORCID: Hare, Alex</t>
         </is>
       </c>
     </row>
@@ -5144,12 +5144,12 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Korver, Maartje</t>
+          <t>Contact missing ORCID: McInnes, Will</t>
         </is>
       </c>
     </row>
@@ -5159,12 +5159,12 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Evans, Wiley</t>
+          <t>Contact missing ORCID: Monteith, Zach</t>
         </is>
       </c>
     </row>
@@ -5174,12 +5174,12 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Janusson, Carly</t>
+          <t>Contact missing ORCID: Desmarais, Isabelle</t>
         </is>
       </c>
     </row>
@@ -5189,12 +5189,12 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Oliver, Allison A.</t>
+          <t>Contact missing ORCID: Holmes, Keith</t>
         </is>
       </c>
     </row>
@@ -5204,12 +5204,12 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Hare, Alex</t>
+          <t>Contact missing ORCID: Burt, Jenn</t>
         </is>
       </c>
     </row>
@@ -5219,12 +5219,12 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Giesbrecht, Ian</t>
+          <t>Contact missing ORCID: Floyd, William C.</t>
         </is>
       </c>
     </row>
@@ -5234,12 +5234,12 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Evans, Wiley</t>
+          <t>Contact missing ORCID: Tank, Suzanne E.</t>
         </is>
       </c>
     </row>
@@ -5249,12 +5249,12 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Menounos, Brian</t>
+          <t>Contact missing ORCID: Holmes, Keith</t>
         </is>
       </c>
     </row>
@@ -5264,12 +5264,12 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>a8f61379-14f9-4ccc-bc9b-4408ba8340d7</t>
+          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Opie, Rumer</t>
+          <t>Contact missing ORCID: Viner, Nick</t>
         </is>
       </c>
     </row>
@@ -5279,12 +5279,12 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>c06cb551-351c-456f-8d0c-c8aab9aec162</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Oliver, Allison A.</t>
+          <t>Contact missing ORCID: Floyd, William C.</t>
         </is>
       </c>
     </row>
@@ -5294,355 +5294,10 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Barrette, Jessy</t>
-        </is>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="n">
-        <v>325</v>
-      </c>
-      <c r="B327" t="inlineStr">
-        <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
-        </is>
-      </c>
-      <c r="C327" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Godwin, Sean</t>
-        </is>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="n">
-        <v>326</v>
-      </c>
-      <c r="B328" t="inlineStr">
-        <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
-        </is>
-      </c>
-      <c r="C328" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Krkosek, Martin</t>
-        </is>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="n">
-        <v>327</v>
-      </c>
-      <c r="B329" t="inlineStr">
-        <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
-        </is>
-      </c>
-      <c r="C329" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Rogers, Luke A.</t>
-        </is>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="n">
-        <v>328</v>
-      </c>
-      <c r="B330" t="inlineStr">
-        <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
-        </is>
-      </c>
-      <c r="C330" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: McInnes, Will</t>
-        </is>
-      </c>
-    </row>
-    <row r="331">
-      <c r="A331" t="n">
-        <v>329</v>
-      </c>
-      <c r="B331" t="inlineStr">
-        <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
-        </is>
-      </c>
-      <c r="C331" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Savage, Rosie</t>
-        </is>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="n">
-        <v>330</v>
-      </c>
-      <c r="B332" t="inlineStr">
-        <is>
-          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
-        </is>
-      </c>
-      <c r="C332" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Hunt, Brian</t>
-        </is>
-      </c>
-    </row>
-    <row r="333">
-      <c r="A333" t="n">
-        <v>331</v>
-      </c>
-      <c r="B333" t="inlineStr">
-        <is>
-          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
-        </is>
-      </c>
-      <c r="C333" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Haughton, Emily</t>
-        </is>
-      </c>
-    </row>
-    <row r="334">
-      <c r="A334" t="n">
-        <v>332</v>
-      </c>
-      <c r="B334" t="inlineStr">
-        <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
-        </is>
-      </c>
-      <c r="C334" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Korver, Maartje</t>
-        </is>
-      </c>
-    </row>
-    <row r="335">
-      <c r="A335" t="n">
-        <v>333</v>
-      </c>
-      <c r="B335" t="inlineStr">
-        <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
-        </is>
-      </c>
-      <c r="C335" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Holmes, Keith</t>
-        </is>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" t="n">
-        <v>334</v>
-      </c>
-      <c r="B336" t="inlineStr">
-        <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
-        </is>
-      </c>
-      <c r="C336" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Hare, Alex</t>
-        </is>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" t="n">
-        <v>335</v>
-      </c>
-      <c r="B337" t="inlineStr">
-        <is>
-          <t>a9527050-a108-46f7-ac9f-7150b4abede5</t>
-        </is>
-      </c>
-      <c r="C337" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: McInnes, Will</t>
-        </is>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" t="n">
-        <v>336</v>
-      </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
-        </is>
-      </c>
-      <c r="C338" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: McInnes, Will</t>
-        </is>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" t="n">
-        <v>337</v>
-      </c>
-      <c r="B339" t="inlineStr">
-        <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
-        </is>
-      </c>
-      <c r="C339" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Desmarais, Isabelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="n">
-        <v>338</v>
-      </c>
-      <c r="B340" t="inlineStr">
-        <is>
-          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
-        </is>
-      </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Monteith, Zach</t>
-        </is>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" t="n">
-        <v>339</v>
-      </c>
-      <c r="B341" t="inlineStr">
-        <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
-        </is>
-      </c>
-      <c r="C341" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Holmes, Keith</t>
-        </is>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" t="n">
-        <v>340</v>
-      </c>
-      <c r="B342" t="inlineStr">
-        <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
-        </is>
-      </c>
-      <c r="C342" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Burt, Jenn</t>
-        </is>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" t="n">
-        <v>341</v>
-      </c>
-      <c r="B343" t="inlineStr">
-        <is>
-          <t>15f1d4a2-c82a-450c-a8f7-badb34b9c0dc</t>
-        </is>
-      </c>
-      <c r="C343" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Evans, Wiley</t>
-        </is>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="n">
-        <v>342</v>
-      </c>
-      <c r="B344" t="inlineStr">
-        <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
-        </is>
-      </c>
-      <c r="C344" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Floyd, William C.</t>
-        </is>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" t="n">
-        <v>343</v>
-      </c>
-      <c r="B345" t="inlineStr">
-        <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
-        </is>
-      </c>
-      <c r="C345" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Tank, Suzanne E.</t>
-        </is>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" t="n">
-        <v>344</v>
-      </c>
-      <c r="B346" t="inlineStr">
-        <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
-        </is>
-      </c>
-      <c r="C346" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Holmes, Keith</t>
-        </is>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" t="n">
-        <v>345</v>
-      </c>
-      <c r="B347" t="inlineStr">
-        <is>
-          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
-        </is>
-      </c>
-      <c r="C347" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Viner, Nick</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" t="n">
-        <v>346</v>
-      </c>
-      <c r="B348" t="inlineStr">
-        <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
-        </is>
-      </c>
-      <c r="C348" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Floyd, William C.</t>
-        </is>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" t="n">
-        <v>347</v>
-      </c>
-      <c r="B349" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C349" t="inlineStr">
         <is>
           <t>Contact missing ORCID: Hare, Alex</t>
         </is>

</xml_diff>

<commit_message>
Deployed cf1e30a72 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C327"/>
+  <dimension ref="A1:C312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,7 +494,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'GeoBC TRIM Program' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'TRIM BC Base Annotations data' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0272fd06-6ac8-48cd-80c9-b6e05f15be0f</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>0272fd06-6ac8-48cd-80c9-b6e05f15be0f</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
+          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/1.566666' (IsVersionOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
+          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://npafc.org/wp-content/uploads/Public-Documents/2018/1790Canada.pdf' (IsSourceOf) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -839,12 +839,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5194/bg-2017-5' (IsPublishedIn) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -959,12 +959,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://hakai-segmentation.readthedocs.io/en/latest/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://hakai-segmentation.readthedocs.io/en/latest/' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>328b062b-3af6-4149-b90f-a85b99dc40eb</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
+          <t>328b062b-3af6-4149-b90f-a85b99dc40eb</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/5n09-aq76' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/5n09-aq76' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://10.21966/5n09-aq76' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Drew Jordison' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier '10.21966/5n09-aq76' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: creator 'Drew Jordison' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Alex Hare' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='High-resolution time series of surface seawater CO2 content from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA' | DataCite='High-resolution record of surface seawater CO2 content from 2016-08 to 2019-05 from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA (NCEI Accession 0246099)'</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Katie Pocock' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: title CKAN='High-resolution time series of surface seawater CO2 content from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA' | DataCite='High-resolution record of surface seawater CO2 content from 2016-08 to 2019-05 from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA (NCEI Accession 0246099)'</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Katie Campbell' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Katie Pocock' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/pk18-z035' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Katie Campbell' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.21966/pk18-z035' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.1029/2025gl115235' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.1029/2025gl115235' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.1029/2025GL115235' (IsPublishedIn) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/2aap-hn61' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/2aap-hn61' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2084,12 +2084,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2099,12 +2099,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d1ae4278b4' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2114,12 +2114,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2129,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -2159,12 +2159,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.48321/d1ae4278b4' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2189,12 +2189,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_jsp' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2234,12 +2234,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2264,12 +2264,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>582c6ff0-029e-44ba-8ba1-d3f2f39f2005</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/1.566666' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2294,12 +2294,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/lno.11538' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2324,12 +2324,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2339,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.1002/lno.11538' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2354,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2399,12 +2399,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2414,12 +2414,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2429,12 +2429,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2444,12 +2444,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2459,12 +2459,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2474,12 +2474,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2489,12 +2489,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2504,12 +2504,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2519,12 +2519,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -2549,12 +2549,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2564,12 +2564,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2579,12 +2579,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
         </is>
       </c>
     </row>
@@ -2594,12 +2594,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -2639,12 +2639,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2654,12 +2654,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/cqrt-sk09' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2684,12 +2684,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://10.21966/cqrt-sk09' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2714,12 +2714,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2729,12 +2729,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2744,12 +2744,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/1.566666' (Continues) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.14288/1.0396439' (IsSourceOf) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2774,12 +2774,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2789,12 +2789,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2819,12 +2819,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2849,12 +2849,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2864,12 +2864,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2879,12 +2879,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2894,12 +2894,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2909,12 +2909,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2954,12 +2954,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -2984,12 +2984,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2999,12 +2999,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
+          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -3029,12 +3029,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3074,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -3104,12 +3104,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3134,12 +3134,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3149,12 +3149,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3194,12 +3194,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3209,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3224,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -3239,12 +3239,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3284,12 +3284,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3314,12 +3314,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3434,12 +3434,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3449,12 +3449,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3494,12 +3494,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -3554,12 +3554,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3569,12 +3569,12 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3584,12 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -3614,12 +3614,12 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3629,12 +3629,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/xp9x-m243' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3649,7 +3649,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/xp9x-m243' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3659,12 +3659,12 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3704,12 +3704,12 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3719,12 +3719,12 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Emily Haughton' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
         </is>
       </c>
     </row>
@@ -3734,12 +3734,12 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Isabelle Desmarais' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3749,12 +3749,12 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Robert White' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3764,12 +3764,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.1.0' | DataCite='2.0'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3779,12 +3779,12 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3794,12 +3794,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3809,12 +3809,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3824,12 +3824,12 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3839,12 +3839,12 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3854,12 +3854,12 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>2dd906f9-e0fe-4b8c-afe6-c5f2bf7400ae</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3869,12 +3869,12 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3884,12 +3884,12 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2dd906f9-e0fe-4b8c-afe6-c5f2bf7400ae</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.21966/4kr2-jc55' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3899,12 +3899,12 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3914,12 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3929,12 +3929,12 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -3944,12 +3944,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -3974,12 +3974,12 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/4kr2-jc55' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3989,12 +3989,12 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4004,12 +4004,12 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4019,12 +4019,12 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/t8hm-ge90' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4034,12 +4034,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/t8hm-ge90' (Continues) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4049,12 +4049,12 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -4064,12 +4064,12 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -4079,12 +4079,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4094,12 +4094,12 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/t8hm-ge90' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -4109,12 +4109,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/t8hm-ge90' (Continues) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4124,12 +4124,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4139,12 +4139,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'A. A. Oliver' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4154,12 +4154,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4169,12 +4169,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4184,7 +4184,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -4199,12 +4199,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'William C. Floyd' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -4214,12 +4214,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'A. A. Oliver' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4229,12 +4229,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4244,12 +4244,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4259,12 +4259,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4274,12 +4274,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4289,12 +4289,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
+          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4304,12 +4304,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4319,12 +4319,12 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -4334,12 +4334,12 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4349,12 +4349,12 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://10.21966/ytgc-6g46' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4364,12 +4364,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier '10.21966/zjc2-b004' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4379,12 +4379,12 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Maartje C. Korver' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/ytgc-6g46' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4394,12 +4394,12 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'William C. Floyd' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4409,12 +4409,12 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Ray Brunsting' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4424,12 +4424,12 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4439,12 +4439,12 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4454,12 +4454,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/ytgc-6g46' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4469,12 +4469,12 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/zjc2-b004' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4484,12 +4484,12 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/zjc2-b004' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4499,12 +4499,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/ytgc-6g46' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4514,12 +4514,12 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4529,12 +4529,12 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4544,12 +4544,12 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4559,12 +4559,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4574,12 +4574,12 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4589,12 +4589,12 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4604,12 +4604,12 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -4619,12 +4619,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -4634,12 +4634,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -4649,12 +4649,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -4664,12 +4664,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Contact missing ORCID: Korver, Maartje</t>
         </is>
       </c>
     </row>
@@ -4679,12 +4679,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Contact missing ORCID: Oliver, Allison A.</t>
         </is>
       </c>
     </row>
@@ -4694,12 +4694,12 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
+          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing ORCID: Janusson, Carly</t>
         </is>
       </c>
     </row>
@@ -4709,12 +4709,12 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing ORCID: Hare, Alex</t>
         </is>
       </c>
     </row>
@@ -4724,12 +4724,12 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Contact missing ORCID: Giesbrecht, Ian</t>
         </is>
       </c>
     </row>
@@ -4739,12 +4739,12 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Contact missing ORCID: Menounos, Brian</t>
         </is>
       </c>
     </row>
@@ -4754,12 +4754,12 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>a8f61379-14f9-4ccc-bc9b-4408ba8340d7</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing ORCID: Opie, Rumer</t>
         </is>
       </c>
     </row>
@@ -4769,12 +4769,12 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>c06cb551-351c-456f-8d0c-c8aab9aec162</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Contact missing ORCID: Oliver, Allison A.</t>
         </is>
       </c>
     </row>
@@ -4784,12 +4784,12 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: http://catalogue.data.gov.bc.ca/dataset/trim-text-annotation returned status_code=timeout</t>
+          <t>Contact missing ORCID: Godwin, Sean</t>
         </is>
       </c>
     </row>
@@ -4799,12 +4799,12 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Contact missing ORCID: Krkosek, Martin</t>
         </is>
       </c>
     </row>
@@ -4814,12 +4814,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'GeoBC TRIM Program' in DataCite not found in CKAN record</t>
+          <t>Contact missing ORCID: Rogers, Luke A.</t>
         </is>
       </c>
     </row>
@@ -4829,12 +4829,12 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Contact missing ORCID: McInnes, Will</t>
         </is>
       </c>
     </row>
@@ -4844,12 +4844,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'TRIM BC Base Annotations data' in CKAN record not found in DataCite</t>
+          <t>Contact missing ORCID: Savage, Rosie</t>
         </is>
       </c>
     </row>
@@ -4859,12 +4859,12 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
+          <t>Contact missing ORCID: Hunt, Brian</t>
         </is>
       </c>
     </row>
@@ -4874,12 +4874,12 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
+          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
+          <t>Contact missing ORCID: Haughton, Emily</t>
         </is>
       </c>
     </row>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -4904,12 +4904,12 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Oliver, Allison A.</t>
+          <t>Contact missing ORCID: Holmes, Keith</t>
         </is>
       </c>
     </row>
@@ -4919,12 +4919,12 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Janusson, Carly</t>
+          <t>Contact missing ORCID: Hare, Alex</t>
         </is>
       </c>
     </row>
@@ -4934,12 +4934,12 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Hare, Alex</t>
+          <t>Contact missing ORCID: McInnes, Will</t>
         </is>
       </c>
     </row>
@@ -4949,12 +4949,12 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Giesbrecht, Ian</t>
+          <t>Contact missing ORCID: Desmarais, Isabelle</t>
         </is>
       </c>
     </row>
@@ -4964,12 +4964,12 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Menounos, Brian</t>
+          <t>Contact missing ORCID: Monteith, Zach</t>
         </is>
       </c>
     </row>
@@ -4979,12 +4979,12 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>a8f61379-14f9-4ccc-bc9b-4408ba8340d7</t>
+          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Opie, Rumer</t>
+          <t>Contact missing ORCID: Holmes, Keith</t>
         </is>
       </c>
     </row>
@@ -4994,12 +4994,12 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>c06cb551-351c-456f-8d0c-c8aab9aec162</t>
+          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Oliver, Allison A.</t>
+          <t>Contact missing ORCID: Burt, Jenn</t>
         </is>
       </c>
     </row>
@@ -5009,12 +5009,12 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Godwin, Sean</t>
+          <t>Contact missing ORCID: Floyd, William C.</t>
         </is>
       </c>
     </row>
@@ -5024,12 +5024,12 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Krkosek, Martin</t>
+          <t>Contact missing ORCID: Tank, Suzanne E.</t>
         </is>
       </c>
     </row>
@@ -5039,12 +5039,12 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Rogers, Luke A.</t>
+          <t>Contact missing ORCID: Holmes, Keith</t>
         </is>
       </c>
     </row>
@@ -5054,12 +5054,12 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: McInnes, Will</t>
+          <t>Contact missing ORCID: Viner, Nick</t>
         </is>
       </c>
     </row>
@@ -5069,12 +5069,12 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Savage, Rosie</t>
+          <t>Contact missing ORCID: Floyd, William C.</t>
         </is>
       </c>
     </row>
@@ -5084,235 +5084,10 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Hunt, Brian</t>
-        </is>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="n">
-        <v>311</v>
-      </c>
-      <c r="B313" t="inlineStr">
-        <is>
-          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
-        </is>
-      </c>
-      <c r="C313" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Haughton, Emily</t>
-        </is>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" t="n">
-        <v>312</v>
-      </c>
-      <c r="B314" t="inlineStr">
-        <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
-        </is>
-      </c>
-      <c r="C314" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Korver, Maartje</t>
-        </is>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="n">
-        <v>313</v>
-      </c>
-      <c r="B315" t="inlineStr">
-        <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
-        </is>
-      </c>
-      <c r="C315" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Holmes, Keith</t>
-        </is>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="n">
-        <v>314</v>
-      </c>
-      <c r="B316" t="inlineStr">
-        <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
-        </is>
-      </c>
-      <c r="C316" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Hare, Alex</t>
-        </is>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="n">
-        <v>315</v>
-      </c>
-      <c r="B317" t="inlineStr">
-        <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
-        </is>
-      </c>
-      <c r="C317" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: McInnes, Will</t>
-        </is>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="n">
-        <v>316</v>
-      </c>
-      <c r="B318" t="inlineStr">
-        <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
-        </is>
-      </c>
-      <c r="C318" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Desmarais, Isabelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="n">
-        <v>317</v>
-      </c>
-      <c r="B319" t="inlineStr">
-        <is>
-          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
-        </is>
-      </c>
-      <c r="C319" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Monteith, Zach</t>
-        </is>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" t="n">
-        <v>318</v>
-      </c>
-      <c r="B320" t="inlineStr">
-        <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
-        </is>
-      </c>
-      <c r="C320" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Holmes, Keith</t>
-        </is>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="n">
-        <v>319</v>
-      </c>
-      <c r="B321" t="inlineStr">
-        <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
-        </is>
-      </c>
-      <c r="C321" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Burt, Jenn</t>
-        </is>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="n">
-        <v>320</v>
-      </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
-        </is>
-      </c>
-      <c r="C322" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Floyd, William C.</t>
-        </is>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="n">
-        <v>321</v>
-      </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
-        </is>
-      </c>
-      <c r="C323" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Tank, Suzanne E.</t>
-        </is>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="n">
-        <v>322</v>
-      </c>
-      <c r="B324" t="inlineStr">
-        <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
-        </is>
-      </c>
-      <c r="C324" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Holmes, Keith</t>
-        </is>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="n">
-        <v>323</v>
-      </c>
-      <c r="B325" t="inlineStr">
-        <is>
-          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
-        </is>
-      </c>
-      <c r="C325" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Viner, Nick</t>
-        </is>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="n">
-        <v>324</v>
-      </c>
-      <c r="B326" t="inlineStr">
-        <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
-        </is>
-      </c>
-      <c r="C326" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Floyd, William C.</t>
-        </is>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="n">
-        <v>325</v>
-      </c>
-      <c r="B327" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C327" t="inlineStr">
         <is>
           <t>Contact missing ORCID: Hare, Alex</t>
         </is>

</xml_diff>

<commit_message>
Deployed 2998d1d63 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C312"/>
+  <dimension ref="A1:C259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,7 +439,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -449,12 +449,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>ee09830d-dd5e-41eb-8aee-0fe9cef5fe79</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Jenn Burt' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ee09830d-dd5e-41eb-8aee-0fe9cef5fe79</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Jenn Burt' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>0272fd06-6ac8-48cd-80c9-b6e05f15be0f</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'GeoBC TRIM Program' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'TRIM BC Base Annotations data' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0272fd06-6ac8-48cd-80c9-b6e05f15be0f</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -854,12 +854,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5194/bg-2017-5' (IsPublishedIn) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Metadata mismatch: related identifier 'https://hakai-segmentation.readthedocs.io/en/latest/' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -929,12 +929,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -959,12 +959,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>328b062b-3af6-4149-b90f-a85b99dc40eb</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work 'https://10.21966/5n09-aq76' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/5n09-aq76' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
+          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://hakai-segmentation.readthedocs.io/en/latest/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Drew Jordison' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>328b062b-3af6-4149-b90f-a85b99dc40eb</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/5n09-aq76' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/5n09-aq76' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
+          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>e8414189-54c9-4311-874e-b97f9b7916ae</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://huggingface.co/datasets/HakaiInstitute/mussel-seg-1024-1024 returned status_code=429</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Drew Jordison' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: title CKAN='High-resolution time series of surface seawater CO2 content from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA' | DataCite='High-resolution record of surface seawater CO2 content from 2016-08 to 2019-05 from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA (NCEI Accession 0246099)'</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Katie Pocock' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Katie Campbell' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.25921/kmam-ct93' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/pk18-z035' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.1029/2025gl115235' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
+          <t>Metadata mismatch: related identifier '10.1029/2025GL115235' (IsPublishedIn) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='High-resolution time series of surface seawater CO2 content from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA' | DataCite='High-resolution record of surface seawater CO2 content from 2016-08 to 2019-05 from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA (NCEI Accession 0246099)'</t>
+          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Katie Pocock' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Katie Campbell' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/kmam-ct93' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/pk18-z035' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.1029/2025gl115235' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1029/2025GL115235' (IsPublishedIn) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.21966/2aap-hn61' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.21966/9cbv-ra30' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1784,12 +1784,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/2aap-hn61' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.48321/d1ae4278b4' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2069,7 +2069,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2084,12 +2084,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2099,12 +2099,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2114,12 +2114,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2129,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>582c6ff0-029e-44ba-8ba1-d3f2f39f2005</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>Metadata mismatch: related work '10.21966/1.566666' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2159,12 +2159,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d1ae4278b4' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1002/lno.11538' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2174,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2189,12 +2189,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2234,12 +2234,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2264,12 +2264,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2294,12 +2294,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -2324,12 +2324,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2339,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/lno.11538' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2354,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
         </is>
       </c>
     </row>
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -2399,12 +2399,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2414,12 +2414,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2429,12 +2429,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2444,12 +2444,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2459,12 +2459,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
         </is>
       </c>
     </row>
@@ -2474,12 +2474,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work 'https://10.21966/cqrt-sk09' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2489,12 +2489,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2504,12 +2504,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2519,12 +2519,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2549,12 +2549,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2564,12 +2564,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2579,12 +2579,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2594,12 +2594,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2609,12 +2609,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2624,12 +2624,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2639,12 +2639,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2654,12 +2654,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2669,12 +2669,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2684,12 +2684,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/cqrt-sk09' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2714,12 +2714,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2729,12 +2729,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2744,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
+          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -2774,12 +2774,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2789,12 +2789,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2819,12 +2819,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2834,12 +2834,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2849,12 +2849,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2864,12 +2864,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2879,12 +2879,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2894,12 +2894,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2909,12 +2909,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2939,12 +2939,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2954,12 +2954,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -2984,12 +2984,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2999,12 +2999,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3014,12 +3014,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -3044,12 +3044,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3059,12 +3059,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3074,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3089,12 +3089,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/m5rv-4f16' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3104,12 +3104,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -3134,12 +3134,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3149,12 +3149,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3164,12 +3164,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3179,12 +3179,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3194,12 +3194,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3209,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3224,12 +3224,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3239,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3254,7 +3254,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -3269,12 +3269,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3284,12 +3284,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3299,12 +3299,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3314,12 +3314,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3329,12 +3329,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3344,12 +3344,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://10.21966/xp9x-m243' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3359,12 +3359,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3374,12 +3374,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/m5rv-4f16' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
         </is>
       </c>
     </row>
@@ -3389,12 +3389,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3404,12 +3404,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3419,12 +3419,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3434,12 +3434,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3449,12 +3449,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3464,12 +3464,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3494,12 +3494,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3509,12 +3509,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -3539,12 +3539,12 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3554,12 +3554,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/4kr2-jc55' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3569,12 +3569,12 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3584,12 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -3599,12 +3599,12 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3614,12 +3614,12 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3629,12 +3629,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3644,12 +3644,12 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/xp9x-m243' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3659,12 +3659,12 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3674,12 +3674,12 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://10.21966/t8hm-ge90' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3689,12 +3689,12 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier '10.21966/t8hm-ge90' (Continues) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3704,12 +3704,12 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3719,12 +3719,12 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3734,12 +3734,12 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3749,12 +3749,12 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3764,12 +3764,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3779,12 +3779,12 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3794,12 +3794,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3809,12 +3809,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3824,12 +3824,12 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3839,12 +3839,12 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3854,12 +3854,12 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2dd906f9-e0fe-4b8c-afe6-c5f2bf7400ae</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3869,12 +3869,12 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3884,12 +3884,12 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/4kr2-jc55' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3899,12 +3899,12 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://10.21966/ytgc-6g46' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3914,12 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/zjc2-b004' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3929,12 +3929,12 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>Metadata mismatch: related identifier '10.21966/ytgc-6g46' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3944,12 +3944,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3959,12 +3959,12 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3974,12 +3974,12 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3989,12 +3989,12 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4004,12 +4004,12 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4019,12 +4019,12 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/t8hm-ge90' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4034,12 +4034,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/t8hm-ge90' (Continues) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4049,12 +4049,12 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4064,12 +4064,12 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4079,12 +4079,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -4094,12 +4094,12 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4109,12 +4109,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4124,12 +4124,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4139,12 +4139,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'A. A. Oliver' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4154,12 +4154,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -4169,12 +4169,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4184,12 +4184,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -4199,12 +4199,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: http://catalogue.data.gov.bc.ca/dataset/trim-text-annotation returned status_code=timeout</t>
         </is>
       </c>
     </row>
@@ -4214,12 +4214,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4229,12 +4229,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'GeoBC TRIM Program' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -4244,12 +4244,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4259,12 +4259,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'TRIM BC Base Annotations data' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4274,12 +4274,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -4289,807 +4289,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="n">
-        <v>258</v>
-      </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
-        </is>
-      </c>
-      <c r="C260" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="n">
-        <v>259</v>
-      </c>
-      <c r="B261" t="inlineStr">
-        <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
-        </is>
-      </c>
-      <c r="C261" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="n">
-        <v>260</v>
-      </c>
-      <c r="B262" t="inlineStr">
-        <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
-        </is>
-      </c>
-      <c r="C262" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://10.21966/zjc2-b004' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="n">
-        <v>261</v>
-      </c>
-      <c r="B263" t="inlineStr">
-        <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
-        </is>
-      </c>
-      <c r="C263" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://10.21966/ytgc-6g46' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="n">
-        <v>262</v>
-      </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
-        </is>
-      </c>
-      <c r="C264" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier '10.21966/zjc2-b004' (IsPartOf) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="n">
-        <v>263</v>
-      </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
-        </is>
-      </c>
-      <c r="C265" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier '10.21966/ytgc-6g46' (IsPartOf) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="n">
-        <v>264</v>
-      </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C266" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="n">
-        <v>265</v>
-      </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C267" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="n">
-        <v>266</v>
-      </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C268" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="n">
-        <v>267</v>
-      </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
-        </is>
-      </c>
-      <c r="C269" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="n">
-        <v>268</v>
-      </c>
-      <c r="B270" t="inlineStr">
-        <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
-        </is>
-      </c>
-      <c r="C270" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="n">
-        <v>269</v>
-      </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
-        </is>
-      </c>
-      <c r="C271" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="n">
-        <v>270</v>
-      </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C272" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="n">
-        <v>271</v>
-      </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C273" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="n">
-        <v>272</v>
-      </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C274" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="n">
-        <v>273</v>
-      </c>
-      <c r="B275" t="inlineStr">
-        <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
-        </is>
-      </c>
-      <c r="C275" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="n">
-        <v>274</v>
-      </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C276" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="n">
-        <v>275</v>
-      </c>
-      <c r="B277" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C277" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="n">
-        <v>276</v>
-      </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
-        </is>
-      </c>
-      <c r="C278" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="n">
-        <v>277</v>
-      </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C279" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="n">
-        <v>278</v>
-      </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
-        </is>
-      </c>
-      <c r="C280" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="n">
-        <v>279</v>
-      </c>
-      <c r="B281" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C281" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
-        </is>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" t="n">
-        <v>280</v>
-      </c>
-      <c r="B282" t="inlineStr">
-        <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
-        </is>
-      </c>
-      <c r="C282" t="inlineStr">
-        <is>
           <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
-        </is>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" t="n">
-        <v>281</v>
-      </c>
-      <c r="B283" t="inlineStr">
-        <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
-        </is>
-      </c>
-      <c r="C283" t="inlineStr">
-        <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
-        </is>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" t="n">
-        <v>282</v>
-      </c>
-      <c r="B284" t="inlineStr">
-        <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
-        </is>
-      </c>
-      <c r="C284" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Korver, Maartje</t>
-        </is>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285" t="n">
-        <v>283</v>
-      </c>
-      <c r="B285" t="inlineStr">
-        <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
-        </is>
-      </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Oliver, Allison A.</t>
-        </is>
-      </c>
-    </row>
-    <row r="286">
-      <c r="A286" t="n">
-        <v>284</v>
-      </c>
-      <c r="B286" t="inlineStr">
-        <is>
-          <t>f6ad9487-d689-41a3-b610-352224d7759b</t>
-        </is>
-      </c>
-      <c r="C286" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Janusson, Carly</t>
-        </is>
-      </c>
-    </row>
-    <row r="287">
-      <c r="A287" t="n">
-        <v>285</v>
-      </c>
-      <c r="B287" t="inlineStr">
-        <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
-        </is>
-      </c>
-      <c r="C287" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Hare, Alex</t>
-        </is>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="n">
-        <v>286</v>
-      </c>
-      <c r="B288" t="inlineStr">
-        <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
-        </is>
-      </c>
-      <c r="C288" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Giesbrecht, Ian</t>
-        </is>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="n">
-        <v>287</v>
-      </c>
-      <c r="B289" t="inlineStr">
-        <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
-        </is>
-      </c>
-      <c r="C289" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Menounos, Brian</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="n">
-        <v>288</v>
-      </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>a8f61379-14f9-4ccc-bc9b-4408ba8340d7</t>
-        </is>
-      </c>
-      <c r="C290" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Opie, Rumer</t>
-        </is>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="n">
-        <v>289</v>
-      </c>
-      <c r="B291" t="inlineStr">
-        <is>
-          <t>c06cb551-351c-456f-8d0c-c8aab9aec162</t>
-        </is>
-      </c>
-      <c r="C291" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Oliver, Allison A.</t>
-        </is>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="n">
-        <v>290</v>
-      </c>
-      <c r="B292" t="inlineStr">
-        <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
-        </is>
-      </c>
-      <c r="C292" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Godwin, Sean</t>
-        </is>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="n">
-        <v>291</v>
-      </c>
-      <c r="B293" t="inlineStr">
-        <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
-        </is>
-      </c>
-      <c r="C293" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Krkosek, Martin</t>
-        </is>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="n">
-        <v>292</v>
-      </c>
-      <c r="B294" t="inlineStr">
-        <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
-        </is>
-      </c>
-      <c r="C294" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Rogers, Luke A.</t>
-        </is>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="n">
-        <v>293</v>
-      </c>
-      <c r="B295" t="inlineStr">
-        <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
-        </is>
-      </c>
-      <c r="C295" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: McInnes, Will</t>
-        </is>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" t="n">
-        <v>294</v>
-      </c>
-      <c r="B296" t="inlineStr">
-        <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
-        </is>
-      </c>
-      <c r="C296" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Savage, Rosie</t>
-        </is>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" t="n">
-        <v>295</v>
-      </c>
-      <c r="B297" t="inlineStr">
-        <is>
-          <t>2a104224-c3eb-4778-adc3-865b36471b1b</t>
-        </is>
-      </c>
-      <c r="C297" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Hunt, Brian</t>
-        </is>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" t="n">
-        <v>296</v>
-      </c>
-      <c r="B298" t="inlineStr">
-        <is>
-          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
-        </is>
-      </c>
-      <c r="C298" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Haughton, Emily</t>
-        </is>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" t="n">
-        <v>297</v>
-      </c>
-      <c r="B299" t="inlineStr">
-        <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
-        </is>
-      </c>
-      <c r="C299" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Korver, Maartje</t>
-        </is>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" t="n">
-        <v>298</v>
-      </c>
-      <c r="B300" t="inlineStr">
-        <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
-        </is>
-      </c>
-      <c r="C300" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Holmes, Keith</t>
-        </is>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="n">
-        <v>299</v>
-      </c>
-      <c r="B301" t="inlineStr">
-        <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
-        </is>
-      </c>
-      <c r="C301" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Hare, Alex</t>
-        </is>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" t="n">
-        <v>300</v>
-      </c>
-      <c r="B302" t="inlineStr">
-        <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
-        </is>
-      </c>
-      <c r="C302" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: McInnes, Will</t>
-        </is>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" t="n">
-        <v>301</v>
-      </c>
-      <c r="B303" t="inlineStr">
-        <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
-        </is>
-      </c>
-      <c r="C303" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Desmarais, Isabelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="n">
-        <v>302</v>
-      </c>
-      <c r="B304" t="inlineStr">
-        <is>
-          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
-        </is>
-      </c>
-      <c r="C304" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Monteith, Zach</t>
-        </is>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="n">
-        <v>303</v>
-      </c>
-      <c r="B305" t="inlineStr">
-        <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
-        </is>
-      </c>
-      <c r="C305" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Holmes, Keith</t>
-        </is>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="n">
-        <v>304</v>
-      </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
-        </is>
-      </c>
-      <c r="C306" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Burt, Jenn</t>
-        </is>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="n">
-        <v>305</v>
-      </c>
-      <c r="B307" t="inlineStr">
-        <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
-        </is>
-      </c>
-      <c r="C307" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Floyd, William C.</t>
-        </is>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="n">
-        <v>306</v>
-      </c>
-      <c r="B308" t="inlineStr">
-        <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
-        </is>
-      </c>
-      <c r="C308" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Tank, Suzanne E.</t>
-        </is>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="n">
-        <v>307</v>
-      </c>
-      <c r="B309" t="inlineStr">
-        <is>
-          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
-        </is>
-      </c>
-      <c r="C309" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Holmes, Keith</t>
-        </is>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="n">
-        <v>308</v>
-      </c>
-      <c r="B310" t="inlineStr">
-        <is>
-          <t>e1c64faf-88ac-4d28-8144-fad156971b4e</t>
-        </is>
-      </c>
-      <c r="C310" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Viner, Nick</t>
-        </is>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="n">
-        <v>309</v>
-      </c>
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
-        </is>
-      </c>
-      <c r="C311" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Floyd, William C.</t>
-        </is>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="n">
-        <v>310</v>
-      </c>
-      <c r="B312" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C312" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Hare, Alex</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed dff090c63 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C259"/>
+  <dimension ref="A1:C243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
+          <t>0272fd06-6ac8-48cd-80c9-b6e05f15be0f</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0272fd06-6ac8-48cd-80c9-b6e05f15be0f</t>
+          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
+          <t>328b062b-3af6-4149-b90f-a85b99dc40eb</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
+          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>328b062b-3af6-4149-b90f-a85b99dc40eb</t>
+          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/5n09-aq76' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/5n09-aq76' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/5n09-aq76' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/5n09-aq76' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Drew Jordison' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Drew Jordison' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>e8414189-54c9-4311-874e-b97f9b7916ae</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://huggingface.co/datasets/HakaiInstitute/mussel-seg-1024-1024 returned status_code=429</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='High-resolution time series of surface seawater CO2 content from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA' | DataCite='High-resolution record of surface seawater CO2 content from 2016-08 to 2019-05 from the OceansAlaska Shellfish Hatchery in Ketchikan, Alaska, USA (NCEI Accession 0246099)'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Katie Pocock' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Katie Campbell' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/kmam-ct93' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/pk18-z035' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://10.1029/2025gl115235' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.1029/2025GL115235' (IsPublishedIn) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.1029/2025gl115235' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1029/2025GL115235' (IsPublishedIn) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/2aap-hn61' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.21966/9cbv-ra30' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/2aap-hn61' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/9cbv-ra30' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1784,12 +1784,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.48321/d1ae4278b4' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d1ae4278b4' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>582c6ff0-029e-44ba-8ba1-d3f2f39f2005</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.21966/1.566666' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1002/lno.11538' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2084,12 +2084,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2099,12 +2099,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2114,12 +2114,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2129,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>582c6ff0-029e-44ba-8ba1-d3f2f39f2005</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/1.566666' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2159,12 +2159,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/lno.11538' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2174,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2189,12 +2189,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2234,12 +2234,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2264,12 +2264,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
         </is>
       </c>
     </row>
@@ -2294,12 +2294,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2324,12 +2324,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2339,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2354,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
         </is>
       </c>
     </row>
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://10.21966/cqrt-sk09' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2399,12 +2399,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -2429,12 +2429,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2444,12 +2444,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2459,12 +2459,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2474,12 +2474,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/cqrt-sk09' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2489,12 +2489,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2504,12 +2504,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2519,12 +2519,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2549,12 +2549,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2564,12 +2564,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2579,12 +2579,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2594,12 +2594,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2609,12 +2609,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2624,12 +2624,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2639,12 +2639,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2654,12 +2654,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2669,12 +2669,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2684,12 +2684,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2714,12 +2714,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2729,12 +2729,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2744,12 +2744,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2759,12 +2759,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2774,12 +2774,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2789,12 +2789,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2819,12 +2819,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -2849,12 +2849,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2864,12 +2864,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2879,12 +2879,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -2909,12 +2909,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2939,12 +2939,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2954,12 +2954,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2969,12 +2969,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2984,12 +2984,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/m5rv-4f16' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -3029,12 +3029,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3059,12 +3059,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3074,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3089,12 +3089,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/m5rv-4f16' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -3119,12 +3119,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3134,12 +3134,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -3164,12 +3164,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3179,12 +3179,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3194,12 +3194,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3209,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3224,12 +3224,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://10.21966/xp9x-m243' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3239,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3254,12 +3254,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3269,12 +3269,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3284,12 +3284,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
         </is>
       </c>
     </row>
@@ -3299,12 +3299,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3314,12 +3314,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3329,12 +3329,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3344,12 +3344,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/xp9x-m243' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3359,12 +3359,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3374,12 +3374,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3389,12 +3389,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3404,12 +3404,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work '10.21966/4kr2-jc55' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3419,12 +3419,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3434,12 +3434,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3449,12 +3449,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -3464,12 +3464,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3494,12 +3494,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3509,12 +3509,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3524,12 +3524,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://10.21966/t8hm-ge90' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3539,12 +3539,12 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/t8hm-ge90' (Continues) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3554,12 +3554,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/4kr2-jc55' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3569,12 +3569,12 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3584,12 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3599,12 +3599,12 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -3629,12 +3629,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3644,12 +3644,12 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3659,12 +3659,12 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3674,12 +3674,12 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/t8hm-ge90' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3689,12 +3689,12 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/t8hm-ge90' (Continues) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3704,12 +3704,12 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -3734,12 +3734,12 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3749,12 +3749,12 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://10.21966/ytgc-6g46' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3764,12 +3764,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/zjc2-b004' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3779,12 +3779,12 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier '10.21966/ytgc-6g46' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3794,12 +3794,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3809,12 +3809,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/gsbw-bz85 status_code=502</t>
         </is>
       </c>
     </row>
@@ -3824,12 +3824,12 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3839,12 +3839,12 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -3869,12 +3869,12 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3884,12 +3884,12 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/zjc2-b004' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3899,12 +3899,12 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://10.21966/ytgc-6g46' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3914,12 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/zjc2-b004' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3929,12 +3929,12 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>5c162406-4886-4a66-9d9c-12c3d0316e2e</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/ytgc-6g46' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3944,12 +3944,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3959,12 +3959,12 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3974,12 +3974,12 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3989,12 +3989,12 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -4004,12 +4004,12 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -4019,12 +4019,12 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -4034,12 +4034,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -4049,250 +4049,10 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="n">
-        <v>242</v>
-      </c>
-      <c r="B244" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="n">
-        <v>243</v>
-      </c>
-      <c r="B245" t="inlineStr">
-        <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
-        </is>
-      </c>
-      <c r="C245" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.5281/zenodo.8323070' (IsDocumentedBy) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="n">
-        <v>244</v>
-      </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
-        </is>
-      </c>
-      <c r="C246" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="n">
-        <v>245</v>
-      </c>
-      <c r="B247" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C247" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="n">
-        <v>246</v>
-      </c>
-      <c r="B248" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C248" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="n">
-        <v>247</v>
-      </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C249" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="n">
-        <v>248</v>
-      </c>
-      <c r="B250" t="inlineStr">
-        <is>
-          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
-        </is>
-      </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="n">
-        <v>249</v>
-      </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C251" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="n">
-        <v>250</v>
-      </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C252" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="n">
-        <v>251</v>
-      </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C253" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: http://catalogue.data.gov.bc.ca/dataset/trim-text-annotation returned status_code=timeout</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="n">
-        <v>252</v>
-      </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="n">
-        <v>253</v>
-      </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C255" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'GeoBC TRIM Program' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="n">
-        <v>254</v>
-      </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C256" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="n">
-        <v>255</v>
-      </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
-        </is>
-      </c>
-      <c r="C257" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'TRIM BC Base Annotations data' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="n">
-        <v>256</v>
-      </c>
-      <c r="B258" t="inlineStr">
-        <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
-        </is>
-      </c>
-      <c r="C258" t="inlineStr">
-        <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="n">
-        <v>257</v>
-      </c>
-      <c r="B259" t="inlineStr">
-        <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
-        </is>
-      </c>
-      <c r="C259" t="inlineStr">
         <is>
           <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>

</xml_diff>

<commit_message>
Deployed ba15e1314 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -839,12 +839,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
+          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>c4d3a53a-faa2-4c3e-bcd3-cfdb0aef0078</t>
+          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.521066' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
+          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.48321/d16d6f987c' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+          <t>Malformed related work identifier (missing doi.org): https://10.1029/2025GL115235</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.1029/2025GL115235</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>cc016896-78d9-46e8-887d-6c1dd106c0e8</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/e4b8-vp48' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/36hp-7f40' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/2aap-hn61' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/2aap-hn61' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/9cbv-ra30' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/9cbv-ra30' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://books.google.ca/books/about/Marine_Phytoplankton.html?id=_lgVAQAAIAAJ&amp;redir_esc=y' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://www.sciencedirect.com/book/9780126930153/identifying-marine-diatoms-and-dinoflagellates' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/529y-sh57' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://library-archives.canada.ca/eng/services/services-libraries/theses/Pages/item.aspx?idNumber=30361177' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1939,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2234,12 +2234,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
         </is>
       </c>
     </row>
@@ -2249,12 +2249,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2494,7 +2494,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.3389/fmars.2022.968470' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/igarss.2012.6351194' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2554,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2569,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2579,12 +2579,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2594,12 +2594,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2609,12 +2609,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2654,12 +2654,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2684,12 +2684,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2714,12 +2714,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2729,12 +2729,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
+          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2789,12 +2789,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2809,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/4jvz-bv44' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/adbg-d170' (IsVersionOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work '10.21966/4jvz-bv44' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2849,12 +2849,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/adbg-d170' (IsVersionOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2879,7 +2879,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -2894,12 +2894,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2914,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2954,12 +2954,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2969,12 +2969,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2984,12 +2984,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/0xex-r023' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2999,12 +2999,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3014,12 +3014,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3029,12 +3029,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3089,12 +3089,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3104,12 +3104,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3149,12 +3149,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>Malformed related work identifier (missing doi.org): https://10.21966/xp9x-m243</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/xp9x-m243</t>
+          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3179,12 +3179,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/zjc2-b004' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3194,12 +3194,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3209,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3224,12 +3224,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3239,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3254,12 +3254,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3269,12 +3269,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
         </is>
       </c>
     </row>
@@ -3284,12 +3284,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3299,12 +3299,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3349,7 +3349,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1109/pacrim47961.2019.8985053' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3359,12 +3359,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.rse.2021.112317' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3419,12 +3419,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3434,12 +3434,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/kace-2d24' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/kace-2d24' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work '10.21966/g7zf-1v08' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3634,7 +3634,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3649,7 +3649,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed a6c8c9cdb to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C197"/>
+  <dimension ref="A1:C198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -839,12 +839,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Malformed related work identifier (missing doi.org): https://10.21966/5n09-aq76</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/5n09-aq76</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/7RX8-DK31' (Continues) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.1029/2025GL115235</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Malformed related work identifier (missing doi.org): https://10.1029/2025GL115235</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1784,12 +1784,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/cqrt-sk09</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Malformed related work identifier (missing doi.org): https://10.21966/cqrt-sk09</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='1.0.4' | DataCite='1.0.0'</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2159,12 +2159,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -2654,7 +2654,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2684,12 +2684,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2714,12 +2714,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2729,12 +2729,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/qpe8-ay93 status_code=502</t>
         </is>
       </c>
     </row>
@@ -2744,12 +2744,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>Malformed related work identifier (missing doi.org): https://10.21966/xp9x-m243</t>
         </is>
       </c>
     </row>
@@ -2759,12 +2759,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/xp9x-m243</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2774,12 +2774,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2789,12 +2789,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2819,12 +2819,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2834,12 +2834,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
         </is>
       </c>
     </row>
@@ -2849,12 +2849,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -2879,12 +2879,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2894,12 +2894,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2909,12 +2909,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2939,12 +2939,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2954,12 +2954,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2984,12 +2984,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/kace-2d24</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2999,12 +2999,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/t8hm-ge90</t>
+          <t>Malformed related work identifier (missing doi.org): https://10.21966/kace-2d24</t>
         </is>
       </c>
     </row>
@@ -3014,12 +3014,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
+          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Malformed related work identifier (missing doi.org): https://10.21966/t8hm-ge90</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3074,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3094,7 +3094,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3104,12 +3104,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -3134,12 +3134,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
+          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3194,12 +3194,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3229,7 +3229,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3239,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3259,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3269,12 +3269,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -3284,12 +3284,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -3314,12 +3314,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -3329,12 +3329,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -3344,12 +3344,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -3359,10 +3359,25 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>196</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
           <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
+      <c r="C198" t="inlineStr">
         <is>
           <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>

</xml_diff>

<commit_message>
Deployed 805fcced4 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C198"/>
+  <dimension ref="A1:C150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,12 +434,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>ee09830d-dd5e-41eb-8aee-0fe9cef5fe79</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -454,7 +454,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Jenn Burt' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -464,12 +464,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ee09830d-dd5e-41eb-8aee-0fe9cef5fe79</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Jenn Burt' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -839,12 +839,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://hakai-segmentation.readthedocs.io/en/latest/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -929,12 +929,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -959,12 +959,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/5n09-aq76</t>
+          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/7RX8-DK31' (Continues) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.1029/2025GL115235</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0049e274-f23e-448c-b307-14aa3b4e0b4a</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203/' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>8a7cd5ea-e167-419e-a5c3-919acafe8455</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1016/j.rse.2018.06.039' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://ntrs.nasa.gov/citations/20110008482' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.21966/4jvz-bv44' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/adbg-d170' (IsVersionOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/cqrt-sk09</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -2069,7 +2069,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2099,12 +2099,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2114,12 +2114,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2159,12 +2159,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2174,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2189,12 +2189,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -2249,12 +2249,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
         </is>
       </c>
     </row>
@@ -2264,12 +2264,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>dcde7ad3-f54e-4210-ae4e-33db5aac63fe</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -2294,12 +2294,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2324,12 +2324,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2339,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2354,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2399,12 +2399,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -2429,12 +2429,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2444,12 +2444,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/4jvz-bv44' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2459,12 +2459,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/adbg-d170' (IsVersionOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2474,12 +2474,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -2519,12 +2519,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2549,12 +2549,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2564,12 +2564,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2579,12 +2579,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://www.onsetcomp.com/products/data-loggers/mx2203' (IsDocumentedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2594,12 +2594,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2609,12 +2609,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2624,12 +2624,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2639,12 +2639,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -2654,730 +2654,10 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="n">
-        <v>149</v>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="n">
-        <v>150</v>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="n">
-        <v>151</v>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="n">
-        <v>152</v>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="n">
-        <v>153</v>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/qpe8-ay93 status_code=502</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="n">
-        <v>154</v>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>45a45b5d-e45c-453c-9d36-036f69d533ae</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/xp9x-m243</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="n">
-        <v>155</v>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="n">
-        <v>156</v>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="n">
-        <v>157</v>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="n">
-        <v>158</v>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="n">
-        <v>159</v>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="n">
-        <v>160</v>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="n">
-        <v>161</v>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="n">
-        <v>162</v>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="n">
-        <v>163</v>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="n">
-        <v>164</v>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="n">
-        <v>165</v>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="n">
-        <v>166</v>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://github.com/HakaiInstitute/sentinels-light-trap-public/blob/main/docs/Protocols/2024%20Light%20Trap%20Protocols.pdf' (IsDocumentedBy) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="n">
-        <v>167</v>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
-        </is>
-      </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="n">
-        <v>168</v>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
-        </is>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="n">
-        <v>169</v>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="n">
-        <v>170</v>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="n">
-        <v>171</v>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/kace-2d24</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="n">
-        <v>172</v>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>262f25ca-ca11-4b10-bb6c-9aec117319a9</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>Malformed related work identifier (missing doi.org): https://10.21966/t8hm-ge90</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="n">
-        <v>173</v>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>No DOI defined</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="n">
-        <v>174</v>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>bdc6c492-dbb1-4d6e-90b8-d7bddf2c6356</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="n">
-        <v>175</v>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="n">
-        <v>176</v>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="n">
-        <v>177</v>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="n">
-        <v>178</v>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>No DOI defined</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="n">
-        <v>179</v>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="n">
-        <v>180</v>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="n">
-        <v>181</v>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="n">
-        <v>182</v>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="n">
-        <v>183</v>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="n">
-        <v>184</v>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="n">
-        <v>185</v>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="n">
-        <v>186</v>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="n">
-        <v>187</v>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="n">
-        <v>188</v>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="n">
-        <v>189</v>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="n">
-        <v>190</v>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
-        </is>
-      </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="n">
-        <v>191</v>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="n">
-        <v>192</v>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="n">
-        <v>193</v>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="n">
-        <v>194</v>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="n">
-        <v>195</v>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
-        </is>
-      </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>196</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
         <is>
           <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>

</xml_diff>

<commit_message>
Deployed de9691335 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C150"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -929,12 +929,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -959,12 +959,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
+          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>3031aa60-689f-4b94-9dc6-9912cc742431</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>c68b9ec8-9f26-4fb0-9333-79730f4ea1ca</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>151f5813-8d7c-4042-8b7a-a878c814145e</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/74y7-v484 status_code=502</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1784,12 +1784,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (IsDescribedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/4jvz-bv44' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/adbg-d170' (IsVersionOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Primary DOI does not have a Hakai prefix (10.21966/): 10.25921/9vnv-0g64</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2084,12 +2084,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2099,12 +2099,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (Documents) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2129,12 +2129,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2159,12 +2159,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2174,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2189,12 +2189,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2234,12 +2234,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2249,12 +2249,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at Sitka Harbor, Sitka, Alaska, USA (Research)' | DataCite='High-resolution record of surface seawater carbon dioxide (CO2) content, water temperature, sea surface salinity and other parameters collected in Sitka Harbor, Alaska, USA from 2017-06-01 to 2021-04-27 (NCEI Accession 0247208)'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2264,12 +2264,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.25921/9vnv-0g64' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -2294,12 +2294,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2324,12 +2324,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2339,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2354,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -2399,12 +2399,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -2414,250 +2414,10 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="n">
-        <v>133</v>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="n">
-        <v>134</v>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="n">
-        <v>135</v>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="n">
-        <v>136</v>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="n">
-        <v>137</v>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="n">
-        <v>138</v>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="n">
-        <v>139</v>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="n">
-        <v>140</v>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="n">
-        <v>141</v>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="n">
-        <v>142</v>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="n">
-        <v>143</v>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="n">
-        <v>144</v>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="n">
-        <v>145</v>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="n">
-        <v>146</v>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="n">
-        <v>147</v>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="n">
-        <v>148</v>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
         <is>
           <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>

</xml_diff>

<commit_message>
Deployed 51b673265 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -929,12 +929,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>151f5813-8d7c-4042-8b7a-a878c814145e</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/74y7-v484 status_code=502</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1784,12 +1784,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (IsDescribedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (IsDescribedBy) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Primary DOI does not have a Hakai prefix (10.21966/): 10.25921/9vnv-0g64</t>
         </is>
       </c>
     </row>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Primary DOI does not have a Hakai prefix (10.21966/): 10.25921/9vnv-0g64</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2084,12 +2084,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2114,12 +2114,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2174,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2224,7 +2224,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2234,12 +2234,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
+          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2339,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -2399,25 +2399,10 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
-        <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="n">
-        <v>132</v>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
         <is>
           <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>

</xml_diff>

<commit_message>
Deployed c885683a4 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>b276330c-4ee9-476a-979a-cebe52d51db6</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Science' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.48321/D18S8D' (IsDescribedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Primary DOI does not have a Hakai prefix (10.21966/): 10.25921/9vnv-0g64</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Primary DOI does not have a Hakai prefix (10.21966/): 10.25921/9vnv-0g64</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2099,12 +2099,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2114,12 +2114,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2129,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2159,12 +2159,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2174,7 +2174,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -2189,12 +2189,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2204,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2234,12 +2234,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2249,12 +2249,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2264,12 +2264,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -2294,12 +2294,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2324,12 +2324,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>
       </c>
     </row>
@@ -2339,70 +2339,10 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="n">
-        <v>128</v>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="n">
-        <v>129</v>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="n">
-        <v>130</v>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="n">
-        <v>131</v>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
         <is>
           <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
         </is>

</xml_diff>

<commit_message>
Deployed e7db26d76 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -659,7 +659,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -929,12 +929,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1002/eap.1897' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/ns9h-1126 status_code=502</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 97484ef39 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>a0ada4b0-faea-4dcd-b9bf-d7ff212315fb</t>
+          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Maartje Korver' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>69268e35-08ac-4e6d-b489-4bb72ac117b1</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -839,12 +839,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
+          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -884,12 +884,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -929,12 +929,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Oceanographic Mooring Time Series, Rivers Inlet, BC, Canada (Research)' | DataCite='Hakai Mooring Water Properties Timeseries Research'</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1darjhrdmvvzesny0d_8arbos95rkufjr/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1034,12 +1034,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'http://ipt.iobis.org/obiscanada/resource?r=hakai_seagrassdensitysurveys' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/c6xs-y324 status_code=404</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/c6xs-y324</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Debora Obrist' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Phytoplankton Pigment Timeseries from High-Performance Liquid Chromatography for the Northern Salish Sea and Central Coast, BC, Canada (Research)' | DataCite='High performance liquid chromatography phytoplankton pigment timeseries for the northern Salish Sea and central coast, British Columbia'</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>dc84cb4c-ba14-4632-a595-eed526bf9db1</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1784,12 +1784,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/47m7-ev69 status_code=404</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No publisher</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/47m7-ev69</t>
         </is>
       </c>
     </row>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/ns9h-1126 status_code=502</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Primary DOI does not have a Hakai prefix (10.21966/): 10.25921/9vnv-0g64</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing ORCID: Haughton, Emily</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>8dc6dfd7-cda8-4fbf-af6a-dcae7d92ed0e</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Contact missing ORCID: Korver, Maartje</t>
         </is>
       </c>
     </row>
@@ -2069,282 +2069,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>110</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>111</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>112</v>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>113</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="n">
-        <v>114</v>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="n">
-        <v>115</v>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="n">
-        <v>116</v>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>50037e63-bfac-4b7a-8547-56337fe40026</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="n">
-        <v>117</v>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>35dd16d8-20b1-49d5-8c59-9cdc02475cd0</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="n">
-        <v>118</v>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="n">
-        <v>119</v>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="n">
-        <v>120</v>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="n">
-        <v>121</v>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="n">
-        <v>122</v>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="n">
-        <v>123</v>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="n">
-        <v>124</v>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="n">
-        <v>125</v>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="n">
-        <v>126</v>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="n">
-        <v>127</v>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
+          <t>Organization missing ROR: McGill University</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 2af5e55c0 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>4a9b4584-a5ef-4baf-9d4a-bacf8e6a5d1d</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>83f387d2-f77e-4921-af15-e064d87ad01a</t>
+          <t>6a1254e5-3815-4289-ba1c-984fb84dc1fe</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/c6xs-y324 status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/c6xs-y324</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.1371/journal.pone.0271477' (IsDerivedFrom) in DataCite not found in CKAN</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/c6xs-y324 status_code=404</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/c6xs-y324</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>401a599c-d74d-4a44-930a-8c0c90659e92</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1784,12 +1784,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/47m7-ev69 status_code=404</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>No publisher</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/47m7-ev69</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No publisher</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'William Floyd' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'W.C. Floyd' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1919,7 +1919,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Haughton, Emily</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Korver, Maartje</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2069,10 +2069,70 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>No version</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>110</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>111</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
           <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Contact missing ORCID: Haughton, Emily</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>112</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Contact missing ORCID: Korver, Maartje</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>113</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
         <is>
           <t>Organization missing ROR: McGill University</t>
         </is>

</xml_diff>

<commit_message>
Deployed ee21fad5a to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -839,12 +839,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -884,12 +884,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>6a1254e5-3815-4289-ba1c-984fb84dc1fe</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6a1254e5-3815-4289-ba1c-984fb84dc1fe</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -959,12 +959,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/c6xs-y324 status_code=404</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/c6xs-y324</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>401a599c-d74d-4a44-930a-8c0c90659e92</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/c6xs-y324 status_code=404</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/c6xs-y324</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>401a599c-d74d-4a44-930a-8c0c90659e92</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/fcwf-p919 status_code=502</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/36hp-7f40 status_code=502</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>No publisher</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>No publisher</t>
+          <t>Metadata mismatch: creator 'William Floyd' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'William Floyd' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'W.C. Floyd' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'W.C. Floyd' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing ORCID: Haughton, Emily</t>
         </is>
       </c>
     </row>
@@ -2084,12 +2084,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
+          <t>Contact missing ORCID: Korver, Maartje</t>
         </is>
       </c>
     </row>
@@ -2103,36 +2103,6 @@
         </is>
       </c>
       <c r="C113" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Haughton, Emily</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>112</v>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Korver, Maartje</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>113</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
         <is>
           <t>Organization missing ROR: McGill University</t>
         </is>

</xml_diff>

<commit_message>
Deployed 0b4c0552e to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,7 +460,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -475,7 +475,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -490,7 +490,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -520,7 +520,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -535,127 +535,127 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -685,52 +685,52 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -739,43 +739,43 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -790,142 +790,142 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>6a1254e5-3815-4289-ba1c-984fb84dc1fe</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>6a1254e5-3815-4289-ba1c-984fb84dc1fe</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -934,148 +934,148 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1084,58 +1084,58 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/c6xs-y324 status_code=404</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -1144,58 +1144,58 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/c6xs-y324 status_code=404</t>
+          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/c6xs-y324</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>401a599c-d74d-4a44-930a-8c0c90659e92</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/c6xs-y324</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>401a599c-d74d-4a44-930a-8c0c90659e92</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1204,43 +1204,43 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -1249,103 +1249,103 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>61</v>
+        <v>2</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -1354,17 +1354,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1375,11 +1375,11 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1390,52 +1390,52 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>67</v>
+        <v>2</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -1444,58 +1444,58 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>72</v>
+        <v>1</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -1525,41 +1525,41 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1570,11 +1570,11 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1585,37 +1585,37 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/fcwf-p919 status_code=502</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -1624,17 +1624,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -1645,101 +1645,101 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>86</v>
+        <v>2</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -1750,361 +1750,226 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>89</v>
+        <v>0</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>91</v>
+        <v>1</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>357b017c-6add-4bde-95d0-386bdbab92b3</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/36hp-7f40 status_code=502</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>94</v>
+        <v>1</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>No publisher</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>96</v>
+        <v>1</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'William Floyd' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>97</v>
+        <v>2</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'W.C. Floyd' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>101</v>
+        <v>1</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
-        <v>103</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="n">
-        <v>104</v>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
-        <v>105</v>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="n">
-        <v>106</v>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>107</v>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>108</v>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
-        <v>109</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Haughton, Emily</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>110</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Korver, Maartje</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>111</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>Organization missing ROR: McGill University</t>
+          <t>No version</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 780899cbc to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/54tw-kh93 status_code=502</t>
         </is>
       </c>
     </row>
@@ -734,18 +734,18 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -754,13 +754,13 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -769,22 +769,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -839,18 +839,18 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -865,22 +865,22 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -889,22 +889,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6a1254e5-3815-4289-ba1c-984fb84dc1fe</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/1yev-s239 status_code=502</t>
         </is>
       </c>
     </row>
@@ -929,33 +929,33 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>6a1254e5-3815-4289-ba1c-984fb84dc1fe</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -964,37 +964,37 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1034,48 +1034,48 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1084,37 +1084,37 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1124,27 +1124,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/c6xs-y324 status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/c6xs-y324</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1154,48 +1154,48 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>401a599c-d74d-4a44-930a-8c0c90659e92</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/c6xs-y324 status_code=404</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Failed to retrieve DOI from dataCite [404] The resource you are looking for doesn't exist.: 10.21966/c6xs-y324</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>401a599c-d74d-4a44-930a-8c0c90659e92</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1204,43 +1204,43 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -1249,52 +1249,52 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1304,48 +1304,48 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -1354,17 +1354,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1375,11 +1375,11 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1394,33 +1394,33 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>36e9e6ae-a407-456e-8fe2-a3a78b246bf7</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -1429,13 +1429,13 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -1444,22 +1444,22 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1469,27 +1469,27 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1540,16 +1540,16 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1600,7 +1600,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -1609,13 +1609,13 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -1624,37 +1624,37 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1664,27 +1664,27 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1694,33 +1694,33 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -1729,37 +1729,37 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1769,42 +1769,42 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -1825,31 +1825,31 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1874,18 +1874,18 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -1894,37 +1894,37 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,57 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>1</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2168fd41-96d4-4b72-b5ec-0a5c342aad2a</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>0</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
           <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>No version</t>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>No version</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>0</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 2a96a8a3b to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -764,12 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -779,42 +779,42 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -839,12 +839,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -869,27 +869,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -899,37 +899,37 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>6a1254e5-3815-4289-ba1c-984fb84dc1fe</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -940,11 +940,11 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -959,57 +959,57 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1034,72 +1034,72 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/1.243102' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1139,57 +1139,57 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/drive/u/0/folders/0byed_wx-znmaywdqstvzu3yyvee?resourcekey=0-jt0opjbzravotiwtc-7lcw' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/sbyc-d030' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.21966/j99c-9c14' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/47m7-ev69' (IsSourceOf) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1199,132 +1199,132 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>401a599c-d74d-4a44-930a-8c0c90659e92</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Kira Krumhansl' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>401a599c-d74d-4a44-930a-8c0c90659e92</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'K. Krumhansl' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>401a599c-d74d-4a44-930a-8c0c90659e92</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/bw2d-tg65 status_code=502</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -1364,57 +1364,57 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1484,42 +1484,42 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>cd3ca52d-dc83-4501-9e53-7b00c8ab9090</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1574,42 +1574,42 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -1634,57 +1634,57 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
+          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1769,235 +1769,40 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>0</v>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/J99C-9C14' (IsSourceOf) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="n">
-        <v>1</v>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/sbyc-d030' (IsSourceOf) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n">
-        <v>2</v>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.21966/1.243102' (IsSourceOf) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n">
-        <v>3</v>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/drive/u/0/folders/0Byed_WX-ZNMaYWdqSTVzU3YyVEE?resourcekey=0-Jt0OPJbzrAVOTIWtc-7lcw' (IsSourceOf) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="n">
-        <v>0</v>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="n">
-        <v>0</v>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="n">
-        <v>1</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="n">
-        <v>0</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="n">
-        <v>1</v>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="n">
-        <v>2</v>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="n">
-        <v>0</v>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
-        <v>1</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="n">
-        <v>0</v>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
         <is>
           <t>No version</t>
         </is>

</xml_diff>

<commit_message>
Deployed e1a15b1b7 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -599,18 +599,18 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7ed2118f-ecaa-41e4-aa81-911ffa47bf34</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -644,18 +644,18 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -664,22 +664,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -689,18 +689,18 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -709,13 +709,13 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -724,22 +724,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -764,27 +764,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -839,18 +839,18 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -859,37 +859,37 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1yg1ec4-lvj0ut6csylv0p1udmcq-a5xu/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>b9671efe-5980-452b-90f8-f30e4f1bc194</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JzY5ELRe1sIbZdq7wBmAOT1t7Y1dNJ2v/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -929,12 +929,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -944,27 +944,27 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -974,72 +974,72 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Metadata mismatch: title CKAN='Water Level Time Series, Choke Pass, Central Coast, BC, Canada (Provisional)' | DataCite='Water Level measured from a Pressure Tide Gauge Instrument Deployed in Choke Pass on Calvert Island Research'</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>7607322d-6dea-4758-a257-de8353c899c1</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1049,57 +1049,57 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Metadata mismatch: license CKAN='CC-BY-NC-4.0' | DataCite='cc-by-4.0'</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1124,27 +1124,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hecate.hakai.org/auth/access-request.php?ref=10.21966/tqj2-wh77' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1tCkBSbg8viQE8RDHg-0B3K9qfWbKU_Em/view' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1154,42 +1154,42 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1crbcqqcmvk3ibyxufqxgj7yv7s5a2-1y/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1ZgcHBPDNHUNRvoaYmpj-IcbDrtPWoviN/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1210,46 +1210,46 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -1259,42 +1259,42 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1345,31 +1345,31 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1394,72 +1394,72 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>eb02906a-9645-4486-ba14-46d71c581352</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1469,342 +1469,72 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Tula Foundation' in CKAN record not found in DataCite</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>c2b05382-684f-4349-a64b-b20521223574</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Geospatial Technology Team Hakai' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="n">
-        <v>1</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="n">
-        <v>0</v>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>78b2edef-dab3-47a9-93bb-af63dfcd178d</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="n">
-        <v>0</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=1jukkkqR46AAO14Q80XMWzwojRotSkuYS returned status_code=404</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>1</v>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="n">
-        <v>2</v>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>0</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="n">
-        <v>1</v>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Santiago Gonzalez Arriola' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="n">
-        <v>0</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="n">
-        <v>1</v>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Geospatial' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="n">
-        <v>2</v>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>a4e3915d-207e-493d-97ff-c1e6ad6f0ce7</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="n">
-        <v>0</v>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="n">
-        <v>1</v>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="n">
-        <v>0</v>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="n">
-        <v>1</v>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="n">
-        <v>2</v>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>c2b05382-684f-4349-a64b-b20521223574</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="n">
-        <v>0</v>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1vzyfwx7jwwlxw8wosydkfgt7vxydwlan/view' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="n">
-        <v>1</v>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>e67a81ba-0ac5-49bd-a1fe-02b98f79d8a7</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
           <t>Metadata mismatch: related identifier 'https://docs.google.com/document/d/1j4ENgAW_2XtIHzDYbL8u2E5kOK2JkPEBVYdxcuv8NrE/edit?usp=drive_web&amp;ouid=110988987704080303629' (HasMetadata) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="n">
-        <v>0</v>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>79433a1f-ec07-4cd5-a31a-8c2c53069085</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>No version</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 2b5e8ad23 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>550e7acb-0e3f-461f-bd47-8b6ced16bf43</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier '10.1098/rspb.2020.0108' (HasPart) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.maps.arcgis.com/home/webmap/viewer.html?webmap=75ee2603aa5a45068c7e3579796c3aab' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1mt2v_uv78afjp5z_lhi1gu52bqwko4ms/view?usp=drive_link' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1139,18 +1139,18 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -1159,13 +1159,13 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1174,22 +1174,22 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://hakai.org/stories/great-walls-quadra' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/16gyd2kqiddmvnb9u9hmy12qlp8muxsbb/view?usp=sharing' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 37bddc84d to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,7 +460,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -475,7 +475,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -490,7 +490,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -520,7 +520,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -550,7 +550,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -565,52 +565,52 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1269473 returned status_code=500</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -619,22 +619,877 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>No funder</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Tentative dataset should not have a version</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Floyd, William</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Floyd, William</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Whalen, Matthew</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Korver, Maartje C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Floyd, William</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Lertzman, Ken</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Saunders, Sari</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>5576c279-6d3a-4323-8104-0e1040d9906c</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Burt, Jenn</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Closs, Alana</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Manning, Faye</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Whalen, Matthew</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Rechsteiner, Erin</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>a8f61379-14f9-4ccc-bc9b-4408ba8340d7</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>c06cb551-351c-456f-8d0c-c8aab9aec162</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Oliver, Allison</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Hall, Kyle</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Whalen, Matthew</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Floyd, William</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>4f1e8eac-8390-44d8-93d6-9263fc1dfcf9</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Floyd, William</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Tank, Suzanne</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Lertzman, Ken</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Korver, Maartje C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Floyd, William</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Oliver, Allison</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Tank, Suzanne</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>f51d96b5-1827-4aab-b1ce-575faff1fd03</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Korver, Maartje C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Tank, Suzanne</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Evans, Wiley</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Albers, Sam</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Hare, Alex</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Barrette, Jessy</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Jackson, Jennifer</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>9e4a38d6-eb29-44a8-b495-c56ce74a227c</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Hales, Burke</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Whalen, Matthew</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Hall, Kyle</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>967f98cb-131a-421e-bcfd-467cff973b30</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>967f98cb-131a-421e-bcfd-467cff973b30</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>967f98cb-131a-421e-bcfd-467cff973b30</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>6a6908af-8856-431e-8277-458fee82e534</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Hall, Kyle</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>6a6908af-8856-431e-8277-458fee82e534</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>6a6908af-8856-431e-8277-458fee82e534</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Whalen, Matthew</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>6a6908af-8856-431e-8277-458fee82e534</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Oliver, Allison</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Frazer, Gordon W.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed fbd31d594 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,18 +434,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/trim/</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -454,22 +454,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/1.715740 status_code=502</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -614,27 +614,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -644,42 +644,42 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -689,42 +689,42 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (404): https://doi.org/10.21966/adbg-d170</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/fwa/index.html</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/adbg-d170</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -764,57 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>1</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>0</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>0</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Invalid Resource URL: http://catalogue.data.gov.bc.ca/dataset/trim-text-annotation returned status_code=timeout</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 5115015b3 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,27 +434,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/trim/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1269471 returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -464,27 +464,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>39cc31fc-aa41-43f5-bfe7-48ea173b1f1e</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1456220 returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA865652/ returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -614,27 +614,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -644,42 +644,42 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1269473 returned status_code=500</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/adbg-d170</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -734,27 +734,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,147 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: http://catalogue.data.gov.bc.ca/dataset/trim-text-annotation returned status_code=timeout</t>
+          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/fwa/index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>0</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/?term=PRJNA1195080 returned status_code=500</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1232168/ returned status_code=500</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>0</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>0</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://doi.org/10.21966/adbg-d170</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>0</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>0</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2081eb2e-67c5-44b7-b048-aeb2c646f238</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Broken link (500): https://www.ncbi.nlm.nih.gov/bioproject/?term=PRJNA1041876</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>0</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>0</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed db900e481 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,18 +449,18 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1269471 returned status_code=500</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -469,22 +469,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1456220 returned status_code=500</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA865652/ returned status_code=500</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -644,57 +644,57 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1269473 returned status_code=500</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -704,27 +704,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/fwa/index.html</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -734,42 +734,42 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (404): https://doi.org/10.21966/adbg-d170</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/fwa/index.html</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -779,27 +779,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>2081eb2e-67c5-44b7-b048-aeb2c646f238</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/?term=PRJNA1195080 returned status_code=500</t>
+          <t>Broken link (500): https://www.ncbi.nlm.nih.gov/bioproject/?term=PRJNA1041876</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1232168/ returned status_code=500</t>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
         </is>
       </c>
     </row>
@@ -809,100 +809,10 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>0</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Broken link (404): https://doi.org/10.21966/adbg-d170</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>0</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>1</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>0</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>2081eb2e-67c5-44b7-b048-aeb2c646f238</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Broken link (500): https://www.ncbi.nlm.nih.gov/bioproject/?term=PRJNA1041876</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>0</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>0</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>

</xml_diff>

<commit_message>
Deployed 2b3a844f2 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -629,18 +629,18 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -655,22 +655,22 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -679,22 +679,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/fwa/index.html</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/fwa/index.html</t>
+          <t>Broken link (404): https://doi.org/10.21966/adbg-d170</t>
         </is>
       </c>
     </row>
@@ -719,27 +719,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/adbg-d170</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -749,57 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
           <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>0</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed e442e2f4f to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,12 +434,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b646021f-ec59-490b-b43f-8118e20d2ef6</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -449,12 +449,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b646021f-ec59-490b-b43f-8118e20d2ef6</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -464,12 +464,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>b646021f-ec59-490b-b43f-8118e20d2ef6</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>b646021f-ec59-490b-b43f-8118e20d2ef6</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>No publisher</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>b646021f-ec59-490b-b43f-8118e20d2ef6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=1tPLRwEzDRdKZ-vmFmbJNE57iJha_cFsf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>b646021f-ec59-490b-b43f-8118e20d2ef6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Empty resource name</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>b646021f-ec59-490b-b43f-8118e20d2ef6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Empty resource name</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/trim/</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>0026051c-f514-45d2-bb17-bfe1dc53e96c</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>ab883f0c-0f7c-4ef1-a8a4-c67e82020e0b</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Metadata mismatch: version CKAN='3.0' | DataCite='3.1.0'</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>ab883f0c-0f7c-4ef1-a8a4-c67e82020e0b</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Gillian Sadlier-Brown' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>ab883f0c-0f7c-4ef1-a8a4-c67e82020e0b</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: creator 'Margot Hessing-Lewis' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>36624f4e-7444-4489-be2b-f18df5b96343</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>36624f4e-7444-4489-be2b-f18df5b96343</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>36624f4e-7444-4489-be2b-f18df5b96343</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: http://catalogue.data.gov.bc.ca/dataset/trim-text-annotation returned status_code=timeout</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial Technology Team' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Organization missing ROR: Hakai Institute</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Organization missing ROR: University of Victoria</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Reynolds, John</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,792 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Organization missing ROR: Simon Fraser Univeristy</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>806312b3-91f8-4651-8980-044a0ad52698</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: title CKAN='Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018' | DataCite='Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada'</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>806312b3-91f8-4651-8980-044a0ad52698</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>4c558062-0e9b-4f49-8680-15e3ccb11ea5</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>No funder</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>5ec866ea-5a7a-43d4-9ed1-d4d863304f98</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>5ec866ea-5a7a-43d4-9ed1-d4d863304f98</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>5c358eb3-80e8-40ab-b930-524ab8a59abe</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: related identifier '10.21966/nk1v-ca06' (IsPreviousVersionOf) in DataCite not found in CKAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>9001b91c-b03a-45e0-a4ba-ac6e301b515b</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>No projects associated</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>9001b91c-b03a-45e0-a4ba-ac6e301b515b</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>No version</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>9001b91c-b03a-45e0-a4ba-ac6e301b515b</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>No DOI defined</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>9001b91c-b03a-45e0-a4ba-ac6e301b515b</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>No funder</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>9001b91c-b03a-45e0-a4ba-ac6e301b515b</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>3c07678b-082b-4c23-878f-6720715dabed</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>No version</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>3c07678b-082b-4c23-878f-6720715dabed</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>No DOI defined</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>No funder</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>No version</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: title CKAN='Organic Carbon at Land-Ocean Interface - Calvert Island - 2014-2016' | DataCite='Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada'</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: creator 'Allison Oliver' in DataCite not found in CKAN record</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: author 'A. A. Oliver' in CKAN record not found in DataCite</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.1002/lno.11538' (IsSupplementedBy) in DataCite not found in CKAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0ca4de0c-62a4-4349-a780-a07dc17bfe38</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1tbyg1zmw0kxaidpbzglweav8cxp-h8an/view?usp=sharing' in CKAN not found in DataCite</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0ca4de0c-62a4-4349-a780-a07dc17bfe38</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: related identifier 'https://drive.google.com/file/d/1JUAdsck-dNSgC7BrRB-Eif7fs5JbBnOC/view?usp=sharing' (HasMetadata) in DataCite not found in CKAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ed19c0b0-2a18-4380-a281-953fd769de92</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>No projects associated</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ed19c0b0-2a18-4380-a281-953fd769de92</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>No version</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ed19c0b0-2a18-4380-a281-953fd769de92</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>No funder</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ed19c0b0-2a18-4380-a281-953fd769de92</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: author 'Emily Haughton' in CKAN record not found in DataCite</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ed19c0b0-2a18-4380-a281-953fd769de92</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: related identifier '10.21966/wbg6-7z68' (IsNewVersionOf) in DataCite not found in CKAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ab883f0c-0f7c-4ef1-a8a4-c67e82020e0b</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Duplicate DOI shared with another record: 10.21966/rf3y-8j78</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>806312b3-91f8-4651-8980-044a0ad52698</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Duplicate DOI shared with another record: 10.21966/66x5-a210</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Duplicate DOI shared with another record: 10.21966/n0h9-cq15</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Duplicate DOI shared with another record: 10.21966/66x5-a210</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>f51d96b5-1827-4aab-b1ce-575faff1fd03</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Duplicate DOI shared with another record: 10.21966/rf3y-8j78</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>9001b91c-b03a-45e0-a4ba-ac6e301b515b</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Contact missing ORCID: Holmes, Keith</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>9001b91c-b03a-45e0-a4ba-ac6e301b515b</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Contact missing ORCID: Burt, Jenn</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: St. Pierre, Kyra</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Tank, Suzanne</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Jackson, Jennifer</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Lertzman, Ken</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Floyd, William</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>d39d1eb3-878d-4597-a06a-a85c50dfccee</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Korver, Maartje C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ed19c0b0-2a18-4380-a281-953fd769de92</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Contact missing ORCID: Haughton, Emily</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ed19c0b0-2a18-4380-a281-953fd769de92</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Contact missing ORCID: Giesbrecht, Ian</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed b0eaa0872 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -434,18 +434,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/trim/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -454,22 +454,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/54tw-kh93 status_code=502</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='1.3.0' | DataCite='1.4.0'</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>7a9adcca-b0dc-462f-aa3f-9bb9209158be</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='1.2.0' | DataCite='1.3.0'</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
@@ -614,18 +614,18 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -634,28 +634,28 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -664,28 +664,28 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -694,22 +694,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: http://catalogue.data.gov.bc.ca/dataset/trim-text-annotation returned status_code=timeout</t>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed c9a4b0853 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/54tw-kh93 status_code=502</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -614,18 +614,18 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -640,22 +640,22 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -664,28 +664,28 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -700,29 +700,14 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>0</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
         <is>
           <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
         </is>

</xml_diff>

<commit_message>
Deployed e1636a103 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: related work 'https://drive.google.com/drive/u/1/folders/14ewu0zy1prkykoxglimxtnjuht6xyyta' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
@@ -614,18 +614,18 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -634,28 +634,28 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -664,28 +664,28 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -694,22 +694,67 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>22951dd4-a9f7-4f2a-b11d-d50e184dc223</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/36b8-hq30 status_code=502</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>0</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>0</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed fe8e8ad3f to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,18 +524,18 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -544,22 +544,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -715,16 +715,16 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (502): https://doi.org/10.21966/faz2-0m37</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -734,18 +734,18 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -754,22 +754,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,10 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
-        <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>0</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>

</xml_diff>

<commit_message>
Deployed 5c758392b to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,18 +524,18 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -544,22 +544,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA865652/ returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -659,18 +659,18 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -679,28 +679,28 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -709,22 +709,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -734,27 +734,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -764,27 +764,87 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>0</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>0</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/1.15311 status_code=502</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>0</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>0</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 318f083a8 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,18 +434,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/trim/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -454,28 +454,28 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Resource GitHub repository is not under the HakaiInstitute organization: https://github.com/debobrist/avian-sib</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -484,22 +484,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Resource GitHub repository is not under the HakaiInstitute organization: https://github.com/debobrist/subsidized_isl_bird_communities</t>
+          <t>Resource GitHub repository is not under the HakaiInstitute organization: https://github.com/debobrist/avian-sib</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Resource GitHub repository is not under the HakaiInstitute organization: https://github.com/debobrist/subsidized_isl_bird_communities</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,18 +554,18 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -574,13 +574,13 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -589,22 +589,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.25607/OBP-2068' (IsSupplementedBy) in DataCite not found in CKAN</t>
+          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.25607/OBP-2068' (IsSupplementedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Resource GitHub repository is not under the HakaiInstitute organization: https://github.com/debobrist/food-web-ibt</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Resource GitHub repository is not under the HakaiInstitute organization: https://github.com/debobrist/food-web-ibt</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/nwf1-8x95 status_code=502</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -704,57 +704,57 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (429): https://genomegapp.weebly.com</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -764,27 +764,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -839,27 +839,57 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: http://catalogue.data.gov.bc.ca/dataset/trim-text-annotation returned status_code=timeout</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>0</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>0</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 1008949c7 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -554,18 +554,18 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -574,13 +574,13 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -589,22 +589,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.25607/OBP-2068' (IsSupplementedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.25607/OBP-2068' (IsSupplementedBy) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Resource GitHub repository is not under the HakaiInstitute organization: https://github.com/debobrist/food-web-ibt</t>
+          <t>Metadata mismatch: publication year CKAN='2022' | DataCite='2019'</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>b47e53cd-74dd-4580-80d0-260860064f4b</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
+          <t>Resource GitHub repository is not under the HakaiInstitute organization: https://github.com/debobrist/food-web-ibt</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d1d07d48-c909-41b4-8c0f-13238720749c</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/nwf1-8x95 status_code=502</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
         </is>
       </c>
     </row>
@@ -730,16 +730,16 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Broken link (429): https://genomegapp.weebly.com</t>
+          <t>Metadata mismatch: publication year CKAN='2026' | DataCite='2022'</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Metadata mismatch: publication year CKAN='2025' | DataCite='2022'</t>
         </is>
       </c>
     </row>
@@ -839,18 +839,18 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -859,22 +859,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -884,10 +884,40 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: publication year CKAN='2026' | DataCite='2024'</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>0</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>0</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>

</xml_diff>

<commit_message>
Deployed 19e2c4cac to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Metadata mismatch: related identifier 'dx.doi.org/10.17504/protocols.io.eq2lywxwpvx9/v1' (IsSupplementedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'dx.doi.org/10.17504/protocols.io.eq2lywxwpvx9/v1' (IsSupplementedBy) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -914,42 +914,42 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Tentative dataset should not have a version</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -959,12 +959,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -989,27 +989,27 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.pocean.2022.102843' in CKAN not found in DataCite</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -1019,10 +1019,40 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: related work '10.1016/j.pocean.2022.102843' in CKAN not found in DataCite</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>0</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>0</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>

</xml_diff>

<commit_message>
Deployed 99c1d775b to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,33 +539,33 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -574,37 +574,37 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.25607/OBP-2068' (IsSupplementedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.25607/OBP-2068' (IsSupplementedBy) in DataCite not found in CKAN</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -839,12 +839,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -1034,25 +1034,10 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
-        <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>0</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>

</xml_diff>